<commit_message>
add per-person unit test table templates and folder structure
</commit_message>
<xml_diff>
--- a/test-evidence/M8-Nie-Yichong/UT-M8-table.xlsx
+++ b/test-evidence/M8-Nie-Yichong/UT-M8-table.xlsx
@@ -31,7 +31,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -41,11 +41,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="002E75B6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
     <fill>
@@ -80,15 +75,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -524,27 +516,27 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Category name does not exist</t>
+          <t>分类名不存在</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>create("IT", "Information Technology")</t>
+          <t>create("IT","Information Technology")</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Returns Category object with name=IT</t>
+          <t>返回 Category 对象 name=IT</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Category object returned with correct name and description</t>
+          <t>返回创建后的分类对象名称描述正确</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Category object returned: name=IT, description=Information Technology</t>
+          <t>返回对象 name=IT description=Information Technology</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -566,27 +558,27 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Category name already exists</t>
+          <t>分类名已存在</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>create("IT", "duplicate")</t>
+          <t>create("IT","duplicate")</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Throws IllegalArgumentException</t>
+          <t>抛出 IllegalArgumentException</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>IllegalArgumentException is thrown</t>
+          <t>抛出 IllegalArgumentException</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>IllegalArgumentException thrown</t>
+          <t>抛出 IllegalArgumentException</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -596,76 +588,76 @@
       </c>
     </row>
     <row r="4" ht="42" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>UT-M8-S2-01</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr"/>
-      <c r="D4" s="3" t="inlineStr"/>
-      <c r="E4" s="3" t="inlineStr"/>
-      <c r="F4" s="3" t="inlineStr"/>
-      <c r="G4" s="3" t="inlineStr"/>
-      <c r="H4" s="3" t="inlineStr"/>
+      <c r="C4" s="2" t="inlineStr"/>
+      <c r="D4" s="2" t="inlineStr"/>
+      <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr"/>
+      <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr"/>
     </row>
     <row r="5" ht="42" customHeight="1">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>UT-M8-S2-02</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr"/>
-      <c r="D5" s="3" t="inlineStr"/>
-      <c r="E5" s="3" t="inlineStr"/>
-      <c r="F5" s="3" t="inlineStr"/>
-      <c r="G5" s="3" t="inlineStr"/>
-      <c r="H5" s="3" t="inlineStr"/>
+      <c r="C5" s="2" t="inlineStr"/>
+      <c r="D5" s="2" t="inlineStr"/>
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr"/>
+      <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr"/>
     </row>
     <row r="6" ht="42" customHeight="1">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>UT-M8-S3-01</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr"/>
-      <c r="D6" s="3" t="inlineStr"/>
-      <c r="E6" s="3" t="inlineStr"/>
-      <c r="F6" s="3" t="inlineStr"/>
-      <c r="G6" s="3" t="inlineStr"/>
-      <c r="H6" s="3" t="inlineStr"/>
+      <c r="C6" s="2" t="inlineStr"/>
+      <c r="D6" s="2" t="inlineStr"/>
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr"/>
+      <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr"/>
     </row>
     <row r="7" ht="42" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>UT-M8-S3-02</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr"/>
-      <c r="D7" s="3" t="inlineStr"/>
-      <c r="E7" s="3" t="inlineStr"/>
-      <c r="F7" s="3" t="inlineStr"/>
-      <c r="G7" s="3" t="inlineStr"/>
-      <c r="H7" s="3" t="inlineStr"/>
+      <c r="C7" s="2" t="inlineStr"/>
+      <c r="D7" s="2" t="inlineStr"/>
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr"/>
+      <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
update M8 and M9 unit test tables to English
</commit_message>
<xml_diff>
--- a/test-evidence/M8-Nie-Yichong/UT-M8-table.xlsx
+++ b/test-evidence/M8-Nie-Yichong/UT-M8-table.xlsx
@@ -31,7 +31,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -41,6 +41,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="002E75B6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
     <fill>
@@ -75,12 +80,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -516,27 +524,27 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>分类名不存在</t>
+          <t>Category name does not exist</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>create("IT","Information Technology")</t>
+          <t>create("IT", "Information Technology")</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>返回 Category 对象 name=IT</t>
+          <t>Returns Category object with name=IT</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>返回创建后的分类对象名称描述正确</t>
+          <t>Category object returned with correct name and description</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>返回对象 name=IT description=Information Technology</t>
+          <t>Category object returned: name=IT, description=Information Technology</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -558,27 +566,27 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>分类名已存在</t>
+          <t>Category name already exists</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>create("IT","duplicate")</t>
+          <t>create("IT", "duplicate")</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>抛出 IllegalArgumentException</t>
+          <t>Throws IllegalArgumentException</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>抛出 IllegalArgumentException</t>
+          <t>IllegalArgumentException is thrown</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>抛出 IllegalArgumentException</t>
+          <t>IllegalArgumentException thrown</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -588,76 +596,76 @@
       </c>
     </row>
     <row r="4" ht="42" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>UT-M8-S2-01</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr"/>
-      <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="2" t="inlineStr"/>
-      <c r="F4" s="2" t="inlineStr"/>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr"/>
+      <c r="C4" s="3" t="inlineStr"/>
+      <c r="D4" s="3" t="inlineStr"/>
+      <c r="E4" s="3" t="inlineStr"/>
+      <c r="F4" s="3" t="inlineStr"/>
+      <c r="G4" s="3" t="inlineStr"/>
+      <c r="H4" s="3" t="inlineStr"/>
     </row>
     <row r="5" ht="42" customHeight="1">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>UT-M8-S2-02</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr"/>
-      <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr"/>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr"/>
+      <c r="C5" s="3" t="inlineStr"/>
+      <c r="D5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="inlineStr"/>
+      <c r="F5" s="3" t="inlineStr"/>
+      <c r="G5" s="3" t="inlineStr"/>
+      <c r="H5" s="3" t="inlineStr"/>
     </row>
     <row r="6" ht="42" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>UT-M8-S3-01</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr"/>
-      <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr"/>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr"/>
+      <c r="C6" s="3" t="inlineStr"/>
+      <c r="D6" s="3" t="inlineStr"/>
+      <c r="E6" s="3" t="inlineStr"/>
+      <c r="F6" s="3" t="inlineStr"/>
+      <c r="G6" s="3" t="inlineStr"/>
+      <c r="H6" s="3" t="inlineStr"/>
     </row>
     <row r="7" ht="42" customHeight="1">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>UT-M8-S3-02</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr"/>
-      <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr"/>
-      <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="2" t="inlineStr"/>
+      <c r="C7" s="3" t="inlineStr"/>
+      <c r="D7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="inlineStr"/>
+      <c r="F7" s="3" t="inlineStr"/>
+      <c r="G7" s="3" t="inlineStr"/>
+      <c r="H7" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(m8): add audit logging, admin stats API, and sprint3 tests
</commit_message>
<xml_diff>
--- a/test-evidence/M8-Nie-Yichong/UT-M8-table.xlsx
+++ b/test-evidence/M8-Nie-Yichong/UT-M8-table.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\HONOR Download\ChormDownload\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Program\Java\myJava\CPT202\online-project-selection-system\test-evidence\M8-Nie-Yichong\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0815E232-B331-4A59-B7BB-5795A4FA65A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BD9938C-344E-49EB-BB5B-2F549706DCF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="23236" windowHeight="13875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="61">
   <si>
     <t>Test Name/ID</t>
   </si>
@@ -147,6 +147,94 @@
   </si>
   <si>
     <t>IllegalArgumentException</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>UT-M8-S3-03</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Sprint 3</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>UT-M8-S3-04</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>UserRepository, ProjectTopicRepository, and ApplicationRepository are mocked; count() returns 12, 5, and 8 respectively</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Call adminStatsService.getCounts()</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>A Map with userCount=12, topicCount=5, applicationCount=8</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Returned counts match mocked repository totals</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Same as Expected</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>userRepository.count() is stubbed to throw RuntimeException("Simulated DB failure")</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>A RuntimeException is thrown</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Exception propagates; no Map is returned</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>RuntimeException thrown as expected</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>A valid User admin exists with id=42; AuditLogRepository is mocked</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Call auditLogService.log(admin, "USER_STATUS_TOGGLE", "User", 100L)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>auditLogRepository.save(...) is invoked once with correct AuditLog fields</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>One AuditLog row is persisted with matching action, entity type, entity id, and admin</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Captured AuditLog matches Expected</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>admin is null; AuditLogRepository is mocked</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Call auditLogService.log(null, "CATEGORY_DELETE", "Category", 1L)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>No interaction with auditLogRepository (no save)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Silent skip; nothing is persisted</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>verifyNoInteractions holds</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -177,7 +265,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -192,11 +280,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFE2EFDA"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -227,15 +310,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -540,7 +620,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -578,7 +658,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="54" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>8</v>
       </c>
@@ -682,33 +762,109 @@
         <v>36</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="3" t="s">
+    <row r="6" spans="1:8" ht="94.5" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
-      <c r="H6" s="3"/>
+      <c r="C6" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>36</v>
+      </c>
     </row>
-    <row r="7" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="3" t="s">
+    <row r="7" spans="1:8" ht="54" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
-      <c r="H7" s="3"/>
+      <c r="C7" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="54" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="54" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>36</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>

<commit_message>
feat(M8): complete Sprint 2 & 3 admin features and fix test configuration
</commit_message>
<xml_diff>
--- a/test-evidence/M8-Nie-Yichong/UT-M8-table.xlsx
+++ b/test-evidence/M8-Nie-Yichong/UT-M8-table.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Program\Java\myJava\CPT202\online-project-selection-system\test-evidence\M8-Nie-Yichong\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BD9938C-344E-49EB-BB5B-2F549706DCF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67D59F00-1212-47C0-8CA6-3E922C78EAC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="23236" windowHeight="13875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="70">
   <si>
     <t>Test Name/ID</t>
   </si>
@@ -46,195 +46,251 @@
     <t>Test process</t>
   </si>
   <si>
+    <t>IllegalArgumentException thrown as expected</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Pass</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>UT-M8-S3-03</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Sprint 3</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>UT-M8-S3-04</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>UT-M8-S1-01</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
     <t>Sprint 1</t>
-  </si>
-  <si>
-    <t>Category name does not exist</t>
-  </si>
-  <si>
-    <t>create("IT", "Information Technology")</t>
-  </si>
-  <si>
-    <t>Returns Category object with name=IT</t>
-  </si>
-  <si>
-    <t>Category object returned with correct name and description</t>
-  </si>
-  <si>
-    <t>Category object returned: name=IT, description=Information Technology</t>
-  </si>
-  <si>
-    <t>Pass</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Category name "IT" does not exist in DB</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>categoryService.create("IT", "Information Technology")</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Category object with name=IT, description=Information Technology, isActive=true</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Category created and returned with correct name and description</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Category object returned: name=IT, description=Information Technology, isActive=true</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
     <t>UT-M8-S1-02</t>
-  </si>
-  <si>
-    <t>Category name already exists</t>
-  </si>
-  <si>
-    <t>create("IT", "duplicate")</t>
-  </si>
-  <si>
-    <t>Throws IllegalArgumentException</t>
-  </si>
-  <si>
-    <t>IllegalArgumentException is thrown</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Category name "IT" already exists in DB</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>categoryService.create("IT", "duplicate")</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
     <t>IllegalArgumentException thrown</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Duplicate name is rejected with an exception</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
     <t>UT-M8-S2-01</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
     <t>Sprint 2</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>User with status=disabled exists in DB</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>loadUserByUsername("disabled@student.xjtlu.edu.cn")</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>UserDetails with isEnabled()=false</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Disabled account returns UserDetails where isEnabled() is false</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>UserDetails returned: isEnabled()=false, username correct</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
     <t>UT-M8-S2-02</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Admin user id=1 attempts to disable their own account</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>userAdminService.toggleStatus(1L, "admin@test.com")</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Admin cannot disable their own account</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>UT-M8-S2-03</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Active user exists in DB (integration test)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>PUT /api/admin/users/{id}/status → GET /api/admin/users</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Toggle returns status=disabled; list query confirms the same</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Status change is persisted and reflected in subsequent list query</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>status=disabled confirmed in toggle response and user list</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>UT-M8-S2-04</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Category "DuplicateCategory" already exists in DB</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>POST /api/admin/categories {name:"DuplicateCategory"} (2nd request)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>HTTP 400; error="A category with this name already exists."</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Duplicate category name returns 400 Bad Request</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>400 Bad Request with expected error message</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
     <t>UT-M8-S3-01</t>
-  </si>
-  <si>
-    <t>Sprint 3</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Valid admin user object; AuditLogRepository available</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>auditLogService.log(admin, ACTION_USER_STATUS_TOGGLE, ENTITY_USER, 100L)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>AuditLogRepository.save() called once with correct admin, action, entity fields</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>One audit record is written with correct action and entity information</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>save() called once; all fields (admin, actionType, entityType, entityId) correct</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
     <t>UT-M8-S3-02</t>
-  </si>
-  <si>
-    <t>Target user exists and status is active; admin user is authenticated</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Current admin attempts to disable own account</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>toggleStatus(1001L, "admin@test.com")</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>toggleStatus(1L, "admin@test.com")</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Target user status changes from active to disabled</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>IllegalArgumentException is thrown</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Returned UserSummary status = "disabled"</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>IllegalArgumentException thrown as expected</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Pass</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>UserSummary object returned with status="disabled"</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>IllegalArgumentException</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>UT-M8-S3-03</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Sprint 3</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>UT-M8-S3-04</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>UserRepository, ProjectTopicRepository, and ApplicationRepository are mocked; count() returns 12, 5, and 8 respectively</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Call adminStatsService.getCounts()</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>A Map with userCount=12, topicCount=5, applicationCount=8</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Returned counts match mocked repository totals</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Same as Expected</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>userRepository.count() is stubbed to throw RuntimeException("Simulated DB failure")</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>A RuntimeException is thrown</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Exception propagates; no Map is returned</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>RuntimeException thrown as expected</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>A valid User admin exists with id=42; AuditLogRepository is mocked</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Call auditLogService.log(admin, "USER_STATUS_TOGGLE", "User", 100L)</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>auditLogRepository.save(...) is invoked once with correct AuditLog fields</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>One AuditLog row is persisted with matching action, entity type, entity id, and admin</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Captured AuditLog matches Expected</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>admin is null; AuditLogRepository is mocked</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Call auditLogService.log(null, "CATEGORY_DELETE", "Category", 1L)</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>No interaction with auditLogRepository (no save)</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Silent skip; nothing is persisted</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>verifyNoInteractions holds</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Admin parameter is null</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>auditLogService.log(null, ACTION_CATEGORY_DELETE, ENTITY_CATEGORY, 1L)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>No interaction with AuditLogRepository</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Null admin causes the log call to be silently skipped</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>verifyNoInteractions(auditLogRepository) passed</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Project id=1 exists with status=available</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>adminProjectService.forceArchive(1L)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ProjectTopic: status=archived, previousStatus=available</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Project is archived and its original status is preserved in previousStatus</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>status=archived, previousStatus=available returned</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Project id=3 is archived with previousStatus=available</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>adminProjectService.restore(3L)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ProjectTopic: status=available, previousStatus=null</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Archived project is restored to its previous status; previousStatus is cleared</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>status=available, previousStatus=null returned</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -255,6 +311,7 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="宋体"/>
+      <family val="3"/>
       <charset val="134"/>
     </font>
     <font>
@@ -620,7 +677,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -658,212 +715,264 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="54" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="67.5" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="27" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="H3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B3" s="2" t="s">
+    </row>
+    <row r="4" spans="1:8" ht="40.5" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="H4" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B4" s="2" t="s">
+    </row>
+    <row r="5" spans="1:8" ht="40.5" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E5" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="H4" s="2" t="s">
+      <c r="F5" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="40.5" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
         <v>36</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="94.5" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
-        <v>25</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>26</v>
       </c>
       <c r="C6" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="40.5" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
         <v>42</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="54" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
-        <v>27</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>26</v>
       </c>
       <c r="C7" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G7" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="D7" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>50</v>
-      </c>
       <c r="H7" s="2" t="s">
-        <v>36</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="54" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>40</v>
+        <v>11</v>
       </c>
       <c r="C8" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E8" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="F8" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="G8" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="H8" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="40.5" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="G8" s="2" t="s">
+      <c r="B9" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="H8" s="2" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" ht="54" x14ac:dyDescent="0.3">
-      <c r="A9" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="C9" s="2" t="s">
+      <c r="D9" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="E9" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="F9" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="F9" s="2" t="s">
+      <c r="G9" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="G9" s="2" t="s">
+      <c r="H9" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="40.5" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="H9" s="2" t="s">
-        <v>36</v>
+      <c r="D10" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="54" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>